<commit_message>
A file was deleted and modifications were made to the core pipeline and prompt template files.
</commit_message>
<xml_diff>
--- a/data/out/動作確認/invoice-standard.xlsx
+++ b/data/out/動作確認/invoice-standard.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="GeneratedSheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Invoice" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'GeneratedSheet'!$A$1:$AJ$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Invoice'!$A$1:$AH$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,7 +51,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -59,25 +59,105 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <top style="thin"/>
+    </border>
+    <border>
+      <top style="thin"/>
+    </border>
+    <border>
+      <right style="thin"/>
+      <top style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+    </border>
+    <border/>
+    <border>
+      <right style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <right style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -445,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D7:AD45"/>
+  <dimension ref="C7:AH49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.53" customWidth="1" min="1" max="1"/>
@@ -493,51 +573,118 @@
     <row r="5" ht="17.01" customHeight="1"/>
     <row r="6" ht="17.01" customHeight="1"/>
     <row r="7" ht="17.01" customHeight="1">
-      <c r="N7" s="1" t="inlineStr">
+      <c r="O7" s="1" t="inlineStr">
         <is>
           <t>請</t>
         </is>
       </c>
-      <c r="P7" s="1" t="inlineStr">
+      <c r="Q7" s="1" t="inlineStr">
         <is>
           <t>求</t>
         </is>
       </c>
-      <c r="U7" s="1" t="inlineStr">
+      <c r="V7" s="1" t="inlineStr">
         <is>
           <t>書</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17.01" customHeight="1"/>
-    <row r="9" ht="17.01" customHeight="1"/>
-    <row r="10" ht="17.01" customHeight="1"/>
+    <row r="9" ht="17.01" customHeight="1">
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>年</t>
+        </is>
+      </c>
+      <c r="AE9" s="2" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="AH9" s="2" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17.01" customHeight="1">
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="4" t="n"/>
+      <c r="M10" s="4" t="n"/>
+      <c r="N10" s="4" t="n"/>
+      <c r="O10" s="4" t="n"/>
+      <c r="P10" s="4" t="n"/>
+      <c r="Q10" s="4" t="n"/>
+      <c r="R10" s="5" t="n"/>
+      <c r="S10" s="3" t="n"/>
+      <c r="T10" s="4" t="n"/>
+      <c r="U10" s="4" t="n"/>
+      <c r="V10" s="4" t="n"/>
+      <c r="W10" s="4" t="n"/>
+      <c r="X10" s="4" t="n"/>
+      <c r="Y10" s="4" t="n"/>
+      <c r="Z10" s="4" t="n"/>
+      <c r="AA10" s="4" t="n"/>
+      <c r="AB10" s="5" t="n"/>
+    </row>
     <row r="11" ht="17.01" customHeight="1">
-      <c r="N11" s="2" t="inlineStr">
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
+      <c r="J11" s="7" t="n"/>
+      <c r="K11" s="7" t="n"/>
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7" t="n"/>
+      <c r="N11" s="7" t="n"/>
+      <c r="O11" s="8" t="inlineStr">
         <is>
           <t>様</t>
         </is>
       </c>
-      <c r="U11" s="3" t="inlineStr">
+      <c r="P11" s="7" t="n"/>
+      <c r="Q11" s="7" t="n"/>
+      <c r="R11" s="9" t="n"/>
+      <c r="S11" s="6" t="n"/>
+      <c r="T11" s="7" t="n"/>
+      <c r="U11" s="7" t="n"/>
+      <c r="V11" s="10" t="inlineStr">
         <is>
           <t>（会社名）</t>
         </is>
       </c>
+      <c r="W11" s="7" t="n"/>
+      <c r="X11" s="7" t="n"/>
+      <c r="Y11" s="7" t="n"/>
+      <c r="Z11" s="7" t="n"/>
+      <c r="AA11" s="7" t="n"/>
+      <c r="AB11" s="9" t="n"/>
     </row>
     <row r="12" ht="17.01" customHeight="1">
-      <c r="U12" s="3" t="inlineStr">
+      <c r="V12" s="11" t="inlineStr">
         <is>
           <t>〒</t>
         </is>
       </c>
     </row>
     <row r="13" ht="17.01" customHeight="1">
-      <c r="D13" s="3" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>下記のとおりご請求いたします。</t>
         </is>
       </c>
-      <c r="U13" s="3" t="inlineStr">
+      <c r="V13" s="11" t="inlineStr">
         <is>
           <t>（住所）</t>
         </is>
@@ -545,247 +692,1123 @@
     </row>
     <row r="14" ht="17.01" customHeight="1"/>
     <row r="15" ht="17.01" customHeight="1">
-      <c r="E15" s="3" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>（振込先）</t>
         </is>
       </c>
-      <c r="U15" s="3" t="inlineStr">
+      <c r="V15" s="11" t="inlineStr">
         <is>
           <t>TEL.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="17.01" customHeight="1">
-      <c r="E16" s="3" t="inlineStr">
+      <c r="F16" s="11" t="inlineStr">
         <is>
           <t>預金種別：</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>普通</t>
         </is>
       </c>
-      <c r="U16" s="3" t="inlineStr">
+      <c r="V16" s="11" t="inlineStr">
         <is>
           <t>FAX.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="17.01" customHeight="1">
-      <c r="E17" s="3" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>口座番号：</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="K17" s="11" t="inlineStr">
         <is>
           <t>1234567</t>
         </is>
       </c>
-      <c r="Z17" s="3" t="inlineStr">
+      <c r="AA17" s="12" t="inlineStr">
         <is>
           <t>検</t>
         </is>
       </c>
-      <c r="AA17" s="3" t="inlineStr">
+      <c r="AB17" s="13" t="inlineStr">
         <is>
           <t>印</t>
         </is>
       </c>
-      <c r="AD17" s="3" t="inlineStr">
+      <c r="AC17" s="4" t="n"/>
+      <c r="AD17" s="4" t="n"/>
+      <c r="AE17" s="12" t="inlineStr">
         <is>
           <t>担当者印</t>
         </is>
       </c>
+      <c r="AF17" s="4" t="n"/>
+      <c r="AG17" s="4" t="n"/>
+      <c r="AH17" s="5" t="n"/>
     </row>
     <row r="18" ht="17.01" customHeight="1">
-      <c r="E18" s="3" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>口座名義：</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>◯◯株式会社</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="17.01" customHeight="1"/>
+      <c r="AA18" s="14" t="n"/>
+      <c r="AB18" s="15" t="n"/>
+      <c r="AC18" s="15" t="n"/>
+      <c r="AD18" s="15" t="n"/>
+      <c r="AE18" s="14" t="n"/>
+      <c r="AF18" s="15" t="n"/>
+      <c r="AG18" s="15" t="n"/>
+      <c r="AH18" s="16" t="n"/>
+    </row>
+    <row r="19" ht="17.01" customHeight="1">
+      <c r="AA19" s="14" t="n"/>
+      <c r="AB19" s="15" t="n"/>
+      <c r="AC19" s="15" t="n"/>
+      <c r="AD19" s="15" t="n"/>
+      <c r="AE19" s="14" t="n"/>
+      <c r="AF19" s="15" t="n"/>
+      <c r="AG19" s="15" t="n"/>
+      <c r="AH19" s="16" t="n"/>
+    </row>
     <row r="20" ht="17.01" customHeight="1">
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>御請求金額</t>
         </is>
       </c>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="O20" s="18" t="inlineStr">
         <is>
           <t>¥32,400-</t>
         </is>
       </c>
-      <c r="U20" s="3" t="inlineStr">
+      <c r="V20" s="11" t="inlineStr">
         <is>
           <t>（消費税込み）</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="17.01" customHeight="1"/>
+      <c r="AA20" s="14" t="n"/>
+      <c r="AB20" s="15" t="n"/>
+      <c r="AC20" s="15" t="n"/>
+      <c r="AD20" s="15" t="n"/>
+      <c r="AE20" s="14" t="n"/>
+      <c r="AF20" s="15" t="n"/>
+      <c r="AG20" s="15" t="n"/>
+      <c r="AH20" s="16" t="n"/>
+    </row>
+    <row r="21" ht="17.01" customHeight="1">
+      <c r="AA21" s="6" t="n"/>
+      <c r="AB21" s="7" t="n"/>
+      <c r="AC21" s="7" t="n"/>
+      <c r="AD21" s="7" t="n"/>
+      <c r="AE21" s="6" t="n"/>
+      <c r="AF21" s="7" t="n"/>
+      <c r="AG21" s="7" t="n"/>
+      <c r="AH21" s="9" t="n"/>
+    </row>
     <row r="22" ht="17.01" customHeight="1">
-      <c r="J22" s="3" t="inlineStr">
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
+      <c r="J22" s="4" t="n"/>
+      <c r="K22" s="13" t="inlineStr">
         <is>
           <t>名</t>
         </is>
       </c>
-      <c r="P22" s="3" t="inlineStr">
+      <c r="L22" s="4" t="n"/>
+      <c r="M22" s="4" t="n"/>
+      <c r="N22" s="4" t="n"/>
+      <c r="O22" s="4" t="n"/>
+      <c r="P22" s="4" t="n"/>
+      <c r="Q22" s="12" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
-      <c r="U22" s="3" t="inlineStr">
+      <c r="R22" s="4" t="n"/>
+      <c r="S22" s="3" t="n"/>
+      <c r="T22" s="4" t="n"/>
+      <c r="U22" s="4" t="n"/>
+      <c r="V22" s="13" t="inlineStr">
         <is>
           <t>単価</t>
         </is>
       </c>
-      <c r="X22" s="3" t="inlineStr">
+      <c r="W22" s="4" t="n"/>
+      <c r="X22" s="4" t="n"/>
+      <c r="Y22" s="12" t="inlineStr">
         <is>
           <t>金額</t>
         </is>
       </c>
-      <c r="AC22" s="3" t="inlineStr">
+      <c r="Z22" s="4" t="n"/>
+      <c r="AA22" s="4" t="n"/>
+      <c r="AB22" s="3" t="n"/>
+      <c r="AC22" s="4" t="n"/>
+      <c r="AD22" s="13" t="inlineStr">
         <is>
           <t>摘要</t>
         </is>
       </c>
+      <c r="AE22" s="4" t="n"/>
+      <c r="AF22" s="4" t="n"/>
+      <c r="AG22" s="4" t="n"/>
+      <c r="AH22" s="5" t="n"/>
     </row>
     <row r="23" ht="17.01" customHeight="1">
-      <c r="D23" s="3" t="inlineStr">
+      <c r="E23" s="19" t="inlineStr">
         <is>
           <t>洗面台パイプ修理</t>
         </is>
       </c>
-      <c r="P23" s="3" t="inlineStr">
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="15" t="n"/>
+      <c r="N23" s="15" t="n"/>
+      <c r="O23" s="15" t="n"/>
+      <c r="P23" s="15" t="n"/>
+      <c r="Q23" s="14" t="n"/>
+      <c r="R23" s="15" t="n"/>
+      <c r="S23" s="14" t="n"/>
+      <c r="T23" s="15" t="n"/>
+      <c r="U23" s="15" t="n"/>
+      <c r="V23" s="20" t="inlineStr">
+        <is>
+          <t>21,000</t>
+        </is>
+      </c>
+      <c r="W23" s="15" t="n"/>
+      <c r="X23" s="15" t="n"/>
+      <c r="Y23" s="19" t="inlineStr">
+        <is>
+          <t>21,000</t>
+        </is>
+      </c>
+      <c r="Z23" s="15" t="n"/>
+      <c r="AA23" s="15" t="n"/>
+      <c r="AB23" s="21" t="inlineStr">
+        <is>
+          <t>サンプル</t>
+        </is>
+      </c>
+      <c r="AC23" s="15" t="n"/>
+      <c r="AD23" s="15" t="n"/>
+      <c r="AE23" s="15" t="n"/>
+      <c r="AF23" s="15" t="n"/>
+      <c r="AG23" s="15" t="n"/>
+      <c r="AH23" s="16" t="n"/>
+    </row>
+    <row r="24" ht="17.01" customHeight="1">
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="15" t="n"/>
+      <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="15" t="n"/>
+      <c r="N24" s="15" t="n"/>
+      <c r="O24" s="15" t="n"/>
+      <c r="P24" s="15" t="n"/>
+      <c r="Q24" s="14" t="n"/>
+      <c r="R24" s="15" t="n"/>
+      <c r="S24" s="14" t="n"/>
+      <c r="T24" s="15" t="n"/>
+      <c r="U24" s="15" t="n"/>
+      <c r="V24" s="15" t="n"/>
+      <c r="W24" s="15" t="n"/>
+      <c r="X24" s="15" t="n"/>
+      <c r="Y24" s="14" t="n"/>
+      <c r="Z24" s="15" t="n"/>
+      <c r="AA24" s="15" t="n"/>
+      <c r="AB24" s="14" t="n"/>
+      <c r="AC24" s="15" t="n"/>
+      <c r="AD24" s="15" t="n"/>
+      <c r="AE24" s="15" t="n"/>
+      <c r="AF24" s="15" t="n"/>
+      <c r="AG24" s="15" t="n"/>
+      <c r="AH24" s="16" t="n"/>
+    </row>
+    <row r="25" ht="17.01" customHeight="1">
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>清掃一式</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
+      <c r="I25" s="4" t="n"/>
+      <c r="J25" s="4" t="n"/>
+      <c r="K25" s="4" t="n"/>
+      <c r="L25" s="4" t="n"/>
+      <c r="M25" s="4" t="n"/>
+      <c r="N25" s="4" t="n"/>
+      <c r="O25" s="4" t="n"/>
+      <c r="P25" s="4" t="n"/>
+      <c r="Q25" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="U23" s="3" t="inlineStr">
-        <is>
-          <t>21,000</t>
-        </is>
-      </c>
-      <c r="X23" s="3" t="inlineStr">
-        <is>
-          <t>21,000</t>
-        </is>
-      </c>
-      <c r="AA23" s="5" t="inlineStr">
+      <c r="R25" s="4" t="n"/>
+      <c r="S25" s="3" t="n"/>
+      <c r="T25" s="4" t="n"/>
+      <c r="U25" s="4" t="n"/>
+      <c r="V25" s="13" t="inlineStr">
+        <is>
+          <t>9,000</t>
+        </is>
+      </c>
+      <c r="W25" s="4" t="n"/>
+      <c r="X25" s="4" t="n"/>
+      <c r="Y25" s="12" t="inlineStr">
+        <is>
+          <t>9,000</t>
+        </is>
+      </c>
+      <c r="Z25" s="4" t="n"/>
+      <c r="AA25" s="4" t="n"/>
+      <c r="AB25" s="22" t="inlineStr">
         <is>
           <t>サンプル</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="17.01" customHeight="1"/>
-    <row r="25" ht="17.01" customHeight="1">
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>清掃一式</t>
-        </is>
-      </c>
-      <c r="P25" s="3" t="inlineStr">
+      <c r="AC25" s="4" t="n"/>
+      <c r="AD25" s="4" t="n"/>
+      <c r="AE25" s="4" t="n"/>
+      <c r="AF25" s="4" t="n"/>
+      <c r="AG25" s="4" t="n"/>
+      <c r="AH25" s="5" t="n"/>
+    </row>
+    <row r="26" ht="17.01" customHeight="1">
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="4" t="n"/>
+      <c r="J26" s="4" t="n"/>
+      <c r="K26" s="4" t="n"/>
+      <c r="L26" s="4" t="n"/>
+      <c r="M26" s="4" t="n"/>
+      <c r="N26" s="4" t="n"/>
+      <c r="O26" s="4" t="n"/>
+      <c r="P26" s="4" t="n"/>
+      <c r="Q26" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="U25" s="3" t="inlineStr">
-        <is>
-          <t>9,000</t>
-        </is>
-      </c>
-      <c r="X25" s="3" t="inlineStr">
-        <is>
-          <t>9,000</t>
-        </is>
-      </c>
-      <c r="AA25" s="5" t="inlineStr">
-        <is>
-          <t>サンプル</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="17.01" customHeight="1"/>
-    <row r="27" ht="17.01" customHeight="1"/>
-    <row r="28" ht="17.01" customHeight="1"/>
-    <row r="29" ht="17.01" customHeight="1"/>
-    <row r="30" ht="17.01" customHeight="1"/>
-    <row r="31" ht="17.01" customHeight="1"/>
-    <row r="32" ht="17.01" customHeight="1"/>
-    <row r="33" ht="17.01" customHeight="1"/>
-    <row r="34" ht="17.01" customHeight="1"/>
-    <row r="35" ht="17.01" customHeight="1"/>
-    <row r="36" ht="17.01" customHeight="1"/>
-    <row r="37" ht="17.01" customHeight="1"/>
-    <row r="38" ht="17.01" customHeight="1"/>
-    <row r="39" ht="17.01" customHeight="1"/>
-    <row r="40" ht="17.01" customHeight="1"/>
+      <c r="R26" s="4" t="n"/>
+      <c r="S26" s="3" t="n"/>
+      <c r="T26" s="4" t="n"/>
+      <c r="U26" s="4" t="n"/>
+      <c r="V26" s="4" t="n"/>
+      <c r="W26" s="4" t="n"/>
+      <c r="X26" s="4" t="n"/>
+      <c r="Y26" s="3" t="n"/>
+      <c r="Z26" s="4" t="n"/>
+      <c r="AA26" s="4" t="n"/>
+      <c r="AB26" s="3" t="n"/>
+      <c r="AC26" s="4" t="n"/>
+      <c r="AD26" s="4" t="n"/>
+      <c r="AE26" s="4" t="n"/>
+      <c r="AF26" s="4" t="n"/>
+      <c r="AG26" s="4" t="n"/>
+      <c r="AH26" s="5" t="n"/>
+    </row>
+    <row r="27" ht="17.01" customHeight="1">
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
+      <c r="J27" s="4" t="n"/>
+      <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="n"/>
+      <c r="M27" s="4" t="n"/>
+      <c r="N27" s="4" t="n"/>
+      <c r="O27" s="4" t="n"/>
+      <c r="P27" s="4" t="n"/>
+      <c r="Q27" s="3" t="n"/>
+      <c r="R27" s="4" t="n"/>
+      <c r="S27" s="3" t="n"/>
+      <c r="T27" s="4" t="n"/>
+      <c r="U27" s="4" t="n"/>
+      <c r="V27" s="4" t="n"/>
+      <c r="W27" s="4" t="n"/>
+      <c r="X27" s="4" t="n"/>
+      <c r="Y27" s="3" t="n"/>
+      <c r="Z27" s="4" t="n"/>
+      <c r="AA27" s="4" t="n"/>
+      <c r="AB27" s="3" t="n"/>
+      <c r="AC27" s="4" t="n"/>
+      <c r="AD27" s="4" t="n"/>
+      <c r="AE27" s="4" t="n"/>
+      <c r="AF27" s="4" t="n"/>
+      <c r="AG27" s="4" t="n"/>
+      <c r="AH27" s="5" t="n"/>
+    </row>
+    <row r="28" ht="17.01" customHeight="1">
+      <c r="E28" s="14" t="n"/>
+      <c r="F28" s="15" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="15" t="n"/>
+      <c r="I28" s="15" t="n"/>
+      <c r="J28" s="15" t="n"/>
+      <c r="K28" s="15" t="n"/>
+      <c r="L28" s="15" t="n"/>
+      <c r="M28" s="15" t="n"/>
+      <c r="N28" s="15" t="n"/>
+      <c r="O28" s="15" t="n"/>
+      <c r="P28" s="15" t="n"/>
+      <c r="Q28" s="14" t="n"/>
+      <c r="R28" s="15" t="n"/>
+      <c r="S28" s="14" t="n"/>
+      <c r="T28" s="15" t="n"/>
+      <c r="U28" s="15" t="n"/>
+      <c r="V28" s="15" t="n"/>
+      <c r="W28" s="15" t="n"/>
+      <c r="X28" s="15" t="n"/>
+      <c r="Y28" s="14" t="n"/>
+      <c r="Z28" s="15" t="n"/>
+      <c r="AA28" s="15" t="n"/>
+      <c r="AB28" s="14" t="n"/>
+      <c r="AC28" s="15" t="n"/>
+      <c r="AD28" s="15" t="n"/>
+      <c r="AE28" s="15" t="n"/>
+      <c r="AF28" s="15" t="n"/>
+      <c r="AG28" s="15" t="n"/>
+      <c r="AH28" s="16" t="n"/>
+    </row>
+    <row r="29" ht="17.01" customHeight="1">
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="n"/>
+      <c r="J29" s="4" t="n"/>
+      <c r="K29" s="4" t="n"/>
+      <c r="L29" s="4" t="n"/>
+      <c r="M29" s="4" t="n"/>
+      <c r="N29" s="4" t="n"/>
+      <c r="O29" s="4" t="n"/>
+      <c r="P29" s="4" t="n"/>
+      <c r="Q29" s="3" t="n"/>
+      <c r="R29" s="4" t="n"/>
+      <c r="S29" s="3" t="n"/>
+      <c r="T29" s="4" t="n"/>
+      <c r="U29" s="4" t="n"/>
+      <c r="V29" s="4" t="n"/>
+      <c r="W29" s="4" t="n"/>
+      <c r="X29" s="4" t="n"/>
+      <c r="Y29" s="3" t="n"/>
+      <c r="Z29" s="4" t="n"/>
+      <c r="AA29" s="4" t="n"/>
+      <c r="AB29" s="3" t="n"/>
+      <c r="AC29" s="4" t="n"/>
+      <c r="AD29" s="4" t="n"/>
+      <c r="AE29" s="4" t="n"/>
+      <c r="AF29" s="4" t="n"/>
+      <c r="AG29" s="4" t="n"/>
+      <c r="AH29" s="5" t="n"/>
+    </row>
+    <row r="30" ht="17.01" customHeight="1">
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
+      <c r="J30" s="4" t="n"/>
+      <c r="K30" s="4" t="n"/>
+      <c r="L30" s="4" t="n"/>
+      <c r="M30" s="4" t="n"/>
+      <c r="N30" s="4" t="n"/>
+      <c r="O30" s="4" t="n"/>
+      <c r="P30" s="4" t="n"/>
+      <c r="Q30" s="3" t="n"/>
+      <c r="R30" s="4" t="n"/>
+      <c r="S30" s="3" t="n"/>
+      <c r="T30" s="4" t="n"/>
+      <c r="U30" s="4" t="n"/>
+      <c r="V30" s="4" t="n"/>
+      <c r="W30" s="4" t="n"/>
+      <c r="X30" s="4" t="n"/>
+      <c r="Y30" s="3" t="n"/>
+      <c r="Z30" s="4" t="n"/>
+      <c r="AA30" s="4" t="n"/>
+      <c r="AB30" s="3" t="n"/>
+      <c r="AC30" s="4" t="n"/>
+      <c r="AD30" s="4" t="n"/>
+      <c r="AE30" s="4" t="n"/>
+      <c r="AF30" s="4" t="n"/>
+      <c r="AG30" s="4" t="n"/>
+      <c r="AH30" s="5" t="n"/>
+    </row>
+    <row r="31" ht="17.01" customHeight="1">
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="n"/>
+      <c r="K31" s="4" t="n"/>
+      <c r="L31" s="4" t="n"/>
+      <c r="M31" s="4" t="n"/>
+      <c r="N31" s="4" t="n"/>
+      <c r="O31" s="4" t="n"/>
+      <c r="P31" s="4" t="n"/>
+      <c r="Q31" s="3" t="n"/>
+      <c r="R31" s="4" t="n"/>
+      <c r="S31" s="3" t="n"/>
+      <c r="T31" s="4" t="n"/>
+      <c r="U31" s="4" t="n"/>
+      <c r="V31" s="4" t="n"/>
+      <c r="W31" s="4" t="n"/>
+      <c r="X31" s="4" t="n"/>
+      <c r="Y31" s="3" t="n"/>
+      <c r="Z31" s="4" t="n"/>
+      <c r="AA31" s="4" t="n"/>
+      <c r="AB31" s="3" t="n"/>
+      <c r="AC31" s="4" t="n"/>
+      <c r="AD31" s="4" t="n"/>
+      <c r="AE31" s="4" t="n"/>
+      <c r="AF31" s="4" t="n"/>
+      <c r="AG31" s="4" t="n"/>
+      <c r="AH31" s="5" t="n"/>
+    </row>
+    <row r="32" ht="17.01" customHeight="1">
+      <c r="E32" s="14" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="15" t="n"/>
+      <c r="I32" s="15" t="n"/>
+      <c r="J32" s="15" t="n"/>
+      <c r="K32" s="15" t="n"/>
+      <c r="L32" s="15" t="n"/>
+      <c r="M32" s="15" t="n"/>
+      <c r="N32" s="15" t="n"/>
+      <c r="O32" s="15" t="n"/>
+      <c r="P32" s="15" t="n"/>
+      <c r="Q32" s="14" t="n"/>
+      <c r="R32" s="15" t="n"/>
+      <c r="S32" s="14" t="n"/>
+      <c r="T32" s="15" t="n"/>
+      <c r="U32" s="15" t="n"/>
+      <c r="V32" s="15" t="n"/>
+      <c r="W32" s="15" t="n"/>
+      <c r="X32" s="15" t="n"/>
+      <c r="Y32" s="14" t="n"/>
+      <c r="Z32" s="15" t="n"/>
+      <c r="AA32" s="15" t="n"/>
+      <c r="AB32" s="14" t="n"/>
+      <c r="AC32" s="15" t="n"/>
+      <c r="AD32" s="15" t="n"/>
+      <c r="AE32" s="15" t="n"/>
+      <c r="AF32" s="15" t="n"/>
+      <c r="AG32" s="15" t="n"/>
+      <c r="AH32" s="16" t="n"/>
+    </row>
+    <row r="33" ht="17.01" customHeight="1">
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="4" t="n"/>
+      <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="n"/>
+      <c r="I33" s="4" t="n"/>
+      <c r="J33" s="4" t="n"/>
+      <c r="K33" s="4" t="n"/>
+      <c r="L33" s="4" t="n"/>
+      <c r="M33" s="4" t="n"/>
+      <c r="N33" s="4" t="n"/>
+      <c r="O33" s="4" t="n"/>
+      <c r="P33" s="4" t="n"/>
+      <c r="Q33" s="3" t="n"/>
+      <c r="R33" s="4" t="n"/>
+      <c r="S33" s="3" t="n"/>
+      <c r="T33" s="4" t="n"/>
+      <c r="U33" s="4" t="n"/>
+      <c r="V33" s="4" t="n"/>
+      <c r="W33" s="4" t="n"/>
+      <c r="X33" s="4" t="n"/>
+      <c r="Y33" s="3" t="n"/>
+      <c r="Z33" s="4" t="n"/>
+      <c r="AA33" s="4" t="n"/>
+      <c r="AB33" s="3" t="n"/>
+      <c r="AC33" s="4" t="n"/>
+      <c r="AD33" s="4" t="n"/>
+      <c r="AE33" s="4" t="n"/>
+      <c r="AF33" s="4" t="n"/>
+      <c r="AG33" s="4" t="n"/>
+      <c r="AH33" s="5" t="n"/>
+    </row>
+    <row r="34" ht="17.01" customHeight="1">
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
+      <c r="I34" s="4" t="n"/>
+      <c r="J34" s="4" t="n"/>
+      <c r="K34" s="4" t="n"/>
+      <c r="L34" s="4" t="n"/>
+      <c r="M34" s="4" t="n"/>
+      <c r="N34" s="4" t="n"/>
+      <c r="O34" s="4" t="n"/>
+      <c r="P34" s="4" t="n"/>
+      <c r="Q34" s="3" t="n"/>
+      <c r="R34" s="4" t="n"/>
+      <c r="S34" s="3" t="n"/>
+      <c r="T34" s="4" t="n"/>
+      <c r="U34" s="4" t="n"/>
+      <c r="V34" s="4" t="n"/>
+      <c r="W34" s="4" t="n"/>
+      <c r="X34" s="4" t="n"/>
+      <c r="Y34" s="3" t="n"/>
+      <c r="Z34" s="4" t="n"/>
+      <c r="AA34" s="4" t="n"/>
+      <c r="AB34" s="3" t="n"/>
+      <c r="AC34" s="4" t="n"/>
+      <c r="AD34" s="4" t="n"/>
+      <c r="AE34" s="4" t="n"/>
+      <c r="AF34" s="4" t="n"/>
+      <c r="AG34" s="4" t="n"/>
+      <c r="AH34" s="5" t="n"/>
+    </row>
+    <row r="35" ht="17.01" customHeight="1">
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="4" t="n"/>
+      <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="4" t="n"/>
+      <c r="K35" s="4" t="n"/>
+      <c r="L35" s="4" t="n"/>
+      <c r="M35" s="4" t="n"/>
+      <c r="N35" s="4" t="n"/>
+      <c r="O35" s="4" t="n"/>
+      <c r="P35" s="4" t="n"/>
+      <c r="Q35" s="3" t="n"/>
+      <c r="R35" s="4" t="n"/>
+      <c r="S35" s="3" t="n"/>
+      <c r="T35" s="4" t="n"/>
+      <c r="U35" s="4" t="n"/>
+      <c r="V35" s="4" t="n"/>
+      <c r="W35" s="4" t="n"/>
+      <c r="X35" s="4" t="n"/>
+      <c r="Y35" s="3" t="n"/>
+      <c r="Z35" s="4" t="n"/>
+      <c r="AA35" s="4" t="n"/>
+      <c r="AB35" s="3" t="n"/>
+      <c r="AC35" s="4" t="n"/>
+      <c r="AD35" s="4" t="n"/>
+      <c r="AE35" s="4" t="n"/>
+      <c r="AF35" s="4" t="n"/>
+      <c r="AG35" s="4" t="n"/>
+      <c r="AH35" s="5" t="n"/>
+    </row>
+    <row r="36" ht="17.01" customHeight="1">
+      <c r="E36" s="14" t="n"/>
+      <c r="F36" s="15" t="n"/>
+      <c r="G36" s="15" t="n"/>
+      <c r="H36" s="15" t="n"/>
+      <c r="I36" s="15" t="n"/>
+      <c r="J36" s="15" t="n"/>
+      <c r="K36" s="15" t="n"/>
+      <c r="L36" s="15" t="n"/>
+      <c r="M36" s="15" t="n"/>
+      <c r="N36" s="15" t="n"/>
+      <c r="O36" s="15" t="n"/>
+      <c r="P36" s="15" t="n"/>
+      <c r="Q36" s="14" t="n"/>
+      <c r="R36" s="15" t="n"/>
+      <c r="S36" s="14" t="n"/>
+      <c r="T36" s="15" t="n"/>
+      <c r="U36" s="15" t="n"/>
+      <c r="V36" s="15" t="n"/>
+      <c r="W36" s="15" t="n"/>
+      <c r="X36" s="15" t="n"/>
+      <c r="Y36" s="14" t="n"/>
+      <c r="Z36" s="15" t="n"/>
+      <c r="AA36" s="15" t="n"/>
+      <c r="AB36" s="14" t="n"/>
+      <c r="AC36" s="15" t="n"/>
+      <c r="AD36" s="15" t="n"/>
+      <c r="AE36" s="15" t="n"/>
+      <c r="AF36" s="15" t="n"/>
+      <c r="AG36" s="15" t="n"/>
+      <c r="AH36" s="16" t="n"/>
+    </row>
+    <row r="37" ht="17.01" customHeight="1">
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="n"/>
+      <c r="K37" s="4" t="n"/>
+      <c r="L37" s="4" t="n"/>
+      <c r="M37" s="4" t="n"/>
+      <c r="N37" s="4" t="n"/>
+      <c r="O37" s="4" t="n"/>
+      <c r="P37" s="4" t="n"/>
+      <c r="Q37" s="3" t="n"/>
+      <c r="R37" s="4" t="n"/>
+      <c r="S37" s="3" t="n"/>
+      <c r="T37" s="4" t="n"/>
+      <c r="U37" s="4" t="n"/>
+      <c r="V37" s="4" t="n"/>
+      <c r="W37" s="4" t="n"/>
+      <c r="X37" s="4" t="n"/>
+      <c r="Y37" s="3" t="n"/>
+      <c r="Z37" s="4" t="n"/>
+      <c r="AA37" s="4" t="n"/>
+      <c r="AB37" s="3" t="n"/>
+      <c r="AC37" s="4" t="n"/>
+      <c r="AD37" s="4" t="n"/>
+      <c r="AE37" s="4" t="n"/>
+      <c r="AF37" s="4" t="n"/>
+      <c r="AG37" s="4" t="n"/>
+      <c r="AH37" s="5" t="n"/>
+    </row>
+    <row r="38" ht="17.01" customHeight="1">
+      <c r="E38" s="3" t="n"/>
+      <c r="F38" s="4" t="n"/>
+      <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
+      <c r="I38" s="4" t="n"/>
+      <c r="J38" s="4" t="n"/>
+      <c r="K38" s="4" t="n"/>
+      <c r="L38" s="4" t="n"/>
+      <c r="M38" s="4" t="n"/>
+      <c r="N38" s="4" t="n"/>
+      <c r="O38" s="4" t="n"/>
+      <c r="P38" s="4" t="n"/>
+      <c r="Q38" s="3" t="n"/>
+      <c r="R38" s="4" t="n"/>
+      <c r="S38" s="3" t="n"/>
+      <c r="T38" s="4" t="n"/>
+      <c r="U38" s="4" t="n"/>
+      <c r="V38" s="4" t="n"/>
+      <c r="W38" s="4" t="n"/>
+      <c r="X38" s="4" t="n"/>
+      <c r="Y38" s="3" t="n"/>
+      <c r="Z38" s="4" t="n"/>
+      <c r="AA38" s="4" t="n"/>
+      <c r="AB38" s="3" t="n"/>
+      <c r="AC38" s="4" t="n"/>
+      <c r="AD38" s="4" t="n"/>
+      <c r="AE38" s="4" t="n"/>
+      <c r="AF38" s="4" t="n"/>
+      <c r="AG38" s="4" t="n"/>
+      <c r="AH38" s="5" t="n"/>
+    </row>
+    <row r="39" ht="17.01" customHeight="1">
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="4" t="n"/>
+      <c r="G39" s="4" t="n"/>
+      <c r="H39" s="4" t="n"/>
+      <c r="I39" s="4" t="n"/>
+      <c r="J39" s="4" t="n"/>
+      <c r="K39" s="4" t="n"/>
+      <c r="L39" s="4" t="n"/>
+      <c r="M39" s="4" t="n"/>
+      <c r="N39" s="4" t="n"/>
+      <c r="O39" s="4" t="n"/>
+      <c r="P39" s="4" t="n"/>
+      <c r="Q39" s="3" t="n"/>
+      <c r="R39" s="4" t="n"/>
+      <c r="S39" s="3" t="n"/>
+      <c r="T39" s="4" t="n"/>
+      <c r="U39" s="4" t="n"/>
+      <c r="V39" s="4" t="n"/>
+      <c r="W39" s="4" t="n"/>
+      <c r="X39" s="4" t="n"/>
+      <c r="Y39" s="3" t="n"/>
+      <c r="Z39" s="4" t="n"/>
+      <c r="AA39" s="4" t="n"/>
+      <c r="AB39" s="3" t="n"/>
+      <c r="AC39" s="4" t="n"/>
+      <c r="AD39" s="4" t="n"/>
+      <c r="AE39" s="4" t="n"/>
+      <c r="AF39" s="4" t="n"/>
+      <c r="AG39" s="4" t="n"/>
+      <c r="AH39" s="5" t="n"/>
+    </row>
+    <row r="40" ht="17.01" customHeight="1">
+      <c r="E40" s="14" t="n"/>
+      <c r="F40" s="15" t="n"/>
+      <c r="G40" s="15" t="n"/>
+      <c r="H40" s="15" t="n"/>
+      <c r="I40" s="15" t="n"/>
+      <c r="J40" s="15" t="n"/>
+      <c r="K40" s="15" t="n"/>
+      <c r="L40" s="15" t="n"/>
+      <c r="M40" s="15" t="n"/>
+      <c r="N40" s="15" t="n"/>
+      <c r="O40" s="15" t="n"/>
+      <c r="P40" s="15" t="n"/>
+      <c r="Q40" s="14" t="n"/>
+      <c r="R40" s="15" t="n"/>
+      <c r="S40" s="14" t="n"/>
+      <c r="T40" s="15" t="n"/>
+      <c r="U40" s="15" t="n"/>
+      <c r="V40" s="15" t="n"/>
+      <c r="W40" s="15" t="n"/>
+      <c r="X40" s="15" t="n"/>
+      <c r="Y40" s="14" t="n"/>
+      <c r="Z40" s="15" t="n"/>
+      <c r="AA40" s="15" t="n"/>
+      <c r="AB40" s="14" t="n"/>
+      <c r="AC40" s="15" t="n"/>
+      <c r="AD40" s="15" t="n"/>
+      <c r="AE40" s="15" t="n"/>
+      <c r="AF40" s="15" t="n"/>
+      <c r="AG40" s="15" t="n"/>
+      <c r="AH40" s="16" t="n"/>
+    </row>
     <row r="41" ht="17.01" customHeight="1">
-      <c r="L41" s="3" t="inlineStr">
+      <c r="E41" s="3" t="n"/>
+      <c r="F41" s="4" t="n"/>
+      <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
+      <c r="I41" s="4" t="n"/>
+      <c r="J41" s="4" t="n"/>
+      <c r="K41" s="4" t="n"/>
+      <c r="L41" s="4" t="n"/>
+      <c r="M41" s="13" t="inlineStr">
         <is>
           <t>小</t>
         </is>
       </c>
-      <c r="N41" s="3" t="inlineStr">
+      <c r="N41" s="4" t="n"/>
+      <c r="O41" s="13" t="inlineStr">
         <is>
           <t>計</t>
         </is>
       </c>
-      <c r="X41" s="3" t="inlineStr">
+      <c r="P41" s="4" t="n"/>
+      <c r="Q41" s="3" t="n"/>
+      <c r="R41" s="4" t="n"/>
+      <c r="S41" s="3" t="n"/>
+      <c r="T41" s="4" t="n"/>
+      <c r="U41" s="4" t="n"/>
+      <c r="V41" s="4" t="n"/>
+      <c r="W41" s="4" t="n"/>
+      <c r="X41" s="4" t="n"/>
+      <c r="Y41" s="12" t="inlineStr">
         <is>
           <t>30,000</t>
         </is>
       </c>
+      <c r="Z41" s="4" t="n"/>
+      <c r="AA41" s="4" t="n"/>
+      <c r="AB41" s="3" t="n"/>
+      <c r="AC41" s="4" t="n"/>
+      <c r="AD41" s="4" t="n"/>
+      <c r="AE41" s="4" t="n"/>
+      <c r="AF41" s="4" t="n"/>
+      <c r="AG41" s="4" t="n"/>
+      <c r="AH41" s="5" t="n"/>
     </row>
     <row r="42" ht="17.01" customHeight="1">
-      <c r="L42" s="3" t="inlineStr">
+      <c r="E42" s="12" t="inlineStr">
         <is>
           <t>消費税等</t>
         </is>
       </c>
-      <c r="X42" s="3" t="inlineStr">
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="n"/>
+      <c r="J42" s="4" t="n"/>
+      <c r="K42" s="4" t="n"/>
+      <c r="L42" s="4" t="n"/>
+      <c r="M42" s="4" t="n"/>
+      <c r="N42" s="4" t="n"/>
+      <c r="O42" s="4" t="n"/>
+      <c r="P42" s="4" t="n"/>
+      <c r="Q42" s="3" t="n"/>
+      <c r="R42" s="4" t="n"/>
+      <c r="S42" s="3" t="n"/>
+      <c r="T42" s="4" t="n"/>
+      <c r="U42" s="4" t="n"/>
+      <c r="V42" s="4" t="n"/>
+      <c r="W42" s="4" t="n"/>
+      <c r="X42" s="4" t="n"/>
+      <c r="Y42" s="12" t="inlineStr">
         <is>
           <t>2,400</t>
         </is>
       </c>
+      <c r="Z42" s="4" t="n"/>
+      <c r="AA42" s="4" t="n"/>
+      <c r="AB42" s="3" t="n"/>
+      <c r="AC42" s="4" t="n"/>
+      <c r="AD42" s="4" t="n"/>
+      <c r="AE42" s="4" t="n"/>
+      <c r="AF42" s="4" t="n"/>
+      <c r="AG42" s="4" t="n"/>
+      <c r="AH42" s="5" t="n"/>
     </row>
     <row r="43" ht="17.01" customHeight="1">
-      <c r="L43" s="3" t="inlineStr">
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="4" t="n"/>
+      <c r="G43" s="4" t="n"/>
+      <c r="H43" s="4" t="n"/>
+      <c r="I43" s="4" t="n"/>
+      <c r="J43" s="4" t="n"/>
+      <c r="K43" s="4" t="n"/>
+      <c r="L43" s="4" t="n"/>
+      <c r="M43" s="13" t="inlineStr">
         <is>
           <t>合</t>
         </is>
       </c>
-      <c r="N43" s="3" t="inlineStr">
+      <c r="N43" s="4" t="n"/>
+      <c r="O43" s="13" t="inlineStr">
         <is>
           <t>計</t>
         </is>
       </c>
-      <c r="X43" s="3" t="inlineStr">
+      <c r="P43" s="4" t="n"/>
+      <c r="Q43" s="3" t="n"/>
+      <c r="R43" s="4" t="n"/>
+      <c r="S43" s="3" t="n"/>
+      <c r="T43" s="4" t="n"/>
+      <c r="U43" s="4" t="n"/>
+      <c r="V43" s="4" t="n"/>
+      <c r="W43" s="4" t="n"/>
+      <c r="X43" s="4" t="n"/>
+      <c r="Y43" s="12" t="inlineStr">
         <is>
           <t>32,400</t>
         </is>
       </c>
-    </row>
-    <row r="44" ht="17.01" customHeight="1"/>
+      <c r="Z43" s="4" t="n"/>
+      <c r="AA43" s="4" t="n"/>
+      <c r="AB43" s="3" t="n"/>
+      <c r="AC43" s="4" t="n"/>
+      <c r="AD43" s="4" t="n"/>
+      <c r="AE43" s="4" t="n"/>
+      <c r="AF43" s="4" t="n"/>
+      <c r="AG43" s="4" t="n"/>
+      <c r="AH43" s="5" t="n"/>
+    </row>
+    <row r="44" ht="17.01" customHeight="1">
+      <c r="E44" s="14" t="n"/>
+      <c r="F44" s="15" t="n"/>
+      <c r="G44" s="15" t="n"/>
+      <c r="H44" s="15" t="n"/>
+      <c r="I44" s="15" t="n"/>
+      <c r="J44" s="15" t="n"/>
+      <c r="K44" s="15" t="n"/>
+      <c r="L44" s="15" t="n"/>
+      <c r="M44" s="15" t="n"/>
+      <c r="N44" s="15" t="n"/>
+      <c r="O44" s="15" t="n"/>
+      <c r="P44" s="15" t="n"/>
+      <c r="Q44" s="14" t="n"/>
+      <c r="R44" s="15" t="n"/>
+      <c r="S44" s="14" t="n"/>
+      <c r="T44" s="15" t="n"/>
+      <c r="U44" s="15" t="n"/>
+      <c r="V44" s="15" t="n"/>
+      <c r="W44" s="15" t="n"/>
+      <c r="X44" s="15" t="n"/>
+      <c r="Y44" s="14" t="n"/>
+      <c r="Z44" s="15" t="n"/>
+      <c r="AA44" s="15" t="n"/>
+      <c r="AB44" s="14" t="n"/>
+      <c r="AC44" s="15" t="n"/>
+      <c r="AD44" s="15" t="n"/>
+      <c r="AE44" s="15" t="n"/>
+      <c r="AF44" s="15" t="n"/>
+      <c r="AG44" s="15" t="n"/>
+      <c r="AH44" s="16" t="n"/>
+    </row>
     <row r="45" ht="17.01" customHeight="1">
-      <c r="D45" s="3" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>備考：</t>
         </is>
       </c>
-    </row>
-    <row r="46" ht="17.01" customHeight="1"/>
-    <row r="47" ht="17.01" customHeight="1"/>
-    <row r="48" ht="17.01" customHeight="1"/>
-    <row r="49" ht="17.01" customHeight="1"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="4" t="n"/>
+      <c r="K45" s="4" t="n"/>
+      <c r="L45" s="4" t="n"/>
+      <c r="M45" s="4" t="n"/>
+      <c r="N45" s="4" t="n"/>
+      <c r="O45" s="4" t="n"/>
+      <c r="P45" s="4" t="n"/>
+      <c r="Q45" s="3" t="n"/>
+      <c r="R45" s="4" t="n"/>
+      <c r="S45" s="3" t="n"/>
+      <c r="T45" s="4" t="n"/>
+      <c r="U45" s="4" t="n"/>
+      <c r="V45" s="4" t="n"/>
+      <c r="W45" s="4" t="n"/>
+      <c r="X45" s="4" t="n"/>
+      <c r="Y45" s="3" t="n"/>
+      <c r="Z45" s="4" t="n"/>
+      <c r="AA45" s="4" t="n"/>
+      <c r="AB45" s="3" t="n"/>
+      <c r="AC45" s="4" t="n"/>
+      <c r="AD45" s="4" t="n"/>
+      <c r="AE45" s="4" t="n"/>
+      <c r="AF45" s="4" t="n"/>
+      <c r="AG45" s="4" t="n"/>
+      <c r="AH45" s="5" t="n"/>
+    </row>
+    <row r="46" ht="17.01" customHeight="1">
+      <c r="E46" s="14" t="n"/>
+      <c r="F46" s="15" t="n"/>
+      <c r="G46" s="15" t="n"/>
+      <c r="H46" s="15" t="n"/>
+      <c r="I46" s="15" t="n"/>
+      <c r="J46" s="15" t="n"/>
+      <c r="K46" s="15" t="n"/>
+      <c r="L46" s="15" t="n"/>
+      <c r="M46" s="15" t="n"/>
+      <c r="N46" s="15" t="n"/>
+      <c r="O46" s="15" t="n"/>
+      <c r="P46" s="15" t="n"/>
+      <c r="Q46" s="14" t="n"/>
+      <c r="R46" s="15" t="n"/>
+      <c r="S46" s="14" t="n"/>
+      <c r="T46" s="15" t="n"/>
+      <c r="U46" s="15" t="n"/>
+      <c r="V46" s="15" t="n"/>
+      <c r="W46" s="15" t="n"/>
+      <c r="X46" s="15" t="n"/>
+      <c r="Y46" s="14" t="n"/>
+      <c r="Z46" s="15" t="n"/>
+      <c r="AA46" s="15" t="n"/>
+      <c r="AB46" s="14" t="n"/>
+      <c r="AC46" s="15" t="n"/>
+      <c r="AD46" s="15" t="n"/>
+      <c r="AE46" s="15" t="n"/>
+      <c r="AF46" s="15" t="n"/>
+      <c r="AG46" s="15" t="n"/>
+      <c r="AH46" s="16" t="n"/>
+    </row>
+    <row r="47" ht="17.01" customHeight="1">
+      <c r="E47" s="14" t="n"/>
+      <c r="F47" s="15" t="n"/>
+      <c r="G47" s="15" t="n"/>
+      <c r="H47" s="15" t="n"/>
+      <c r="I47" s="15" t="n"/>
+      <c r="J47" s="15" t="n"/>
+      <c r="K47" s="15" t="n"/>
+      <c r="L47" s="15" t="n"/>
+      <c r="M47" s="15" t="n"/>
+      <c r="N47" s="15" t="n"/>
+      <c r="O47" s="15" t="n"/>
+      <c r="P47" s="15" t="n"/>
+      <c r="Q47" s="14" t="n"/>
+      <c r="R47" s="15" t="n"/>
+      <c r="S47" s="14" t="n"/>
+      <c r="T47" s="15" t="n"/>
+      <c r="U47" s="15" t="n"/>
+      <c r="V47" s="15" t="n"/>
+      <c r="W47" s="15" t="n"/>
+      <c r="X47" s="15" t="n"/>
+      <c r="Y47" s="14" t="n"/>
+      <c r="Z47" s="15" t="n"/>
+      <c r="AA47" s="15" t="n"/>
+      <c r="AB47" s="14" t="n"/>
+      <c r="AC47" s="15" t="n"/>
+      <c r="AD47" s="15" t="n"/>
+      <c r="AE47" s="15" t="n"/>
+      <c r="AF47" s="15" t="n"/>
+      <c r="AG47" s="15" t="n"/>
+      <c r="AH47" s="16" t="n"/>
+    </row>
+    <row r="48" ht="17.01" customHeight="1">
+      <c r="E48" s="14" t="n"/>
+      <c r="F48" s="15" t="n"/>
+      <c r="G48" s="15" t="n"/>
+      <c r="H48" s="15" t="n"/>
+      <c r="I48" s="15" t="n"/>
+      <c r="J48" s="15" t="n"/>
+      <c r="K48" s="15" t="n"/>
+      <c r="L48" s="15" t="n"/>
+      <c r="M48" s="15" t="n"/>
+      <c r="N48" s="15" t="n"/>
+      <c r="O48" s="15" t="n"/>
+      <c r="P48" s="15" t="n"/>
+      <c r="Q48" s="14" t="n"/>
+      <c r="R48" s="15" t="n"/>
+      <c r="S48" s="14" t="n"/>
+      <c r="T48" s="15" t="n"/>
+      <c r="U48" s="15" t="n"/>
+      <c r="V48" s="15" t="n"/>
+      <c r="W48" s="15" t="n"/>
+      <c r="X48" s="15" t="n"/>
+      <c r="Y48" s="14" t="n"/>
+      <c r="Z48" s="15" t="n"/>
+      <c r="AA48" s="15" t="n"/>
+      <c r="AB48" s="14" t="n"/>
+      <c r="AC48" s="15" t="n"/>
+      <c r="AD48" s="15" t="n"/>
+      <c r="AE48" s="15" t="n"/>
+      <c r="AF48" s="15" t="n"/>
+      <c r="AG48" s="15" t="n"/>
+      <c r="AH48" s="16" t="n"/>
+    </row>
+    <row r="49" ht="17.01" customHeight="1">
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="7" t="n"/>
+      <c r="G49" s="7" t="n"/>
+      <c r="H49" s="7" t="n"/>
+      <c r="I49" s="7" t="n"/>
+      <c r="J49" s="7" t="n"/>
+      <c r="K49" s="7" t="n"/>
+      <c r="L49" s="7" t="n"/>
+      <c r="M49" s="7" t="n"/>
+      <c r="N49" s="7" t="n"/>
+      <c r="O49" s="7" t="n"/>
+      <c r="P49" s="7" t="n"/>
+      <c r="Q49" s="6" t="n"/>
+      <c r="R49" s="7" t="n"/>
+      <c r="S49" s="6" t="n"/>
+      <c r="T49" s="7" t="n"/>
+      <c r="U49" s="7" t="n"/>
+      <c r="V49" s="7" t="n"/>
+      <c r="W49" s="7" t="n"/>
+      <c r="X49" s="7" t="n"/>
+      <c r="Y49" s="6" t="n"/>
+      <c r="Z49" s="7" t="n"/>
+      <c r="AA49" s="7" t="n"/>
+      <c r="AB49" s="6" t="n"/>
+      <c r="AC49" s="7" t="n"/>
+      <c r="AD49" s="7" t="n"/>
+      <c r="AE49" s="7" t="n"/>
+      <c r="AF49" s="7" t="n"/>
+      <c r="AG49" s="7" t="n"/>
+      <c r="AH49" s="9" t="n"/>
+    </row>
     <row r="50" ht="17.01" customHeight="1"/>
     <row r="51" ht="17.01" customHeight="1"/>
     <row r="52" ht="17.01" customHeight="1"/>
@@ -836,8 +1859,59 @@
     <row r="97" ht="17.01" customHeight="1"/>
     <row r="98" ht="17.01" customHeight="1"/>
     <row r="99" ht="17.01" customHeight="1"/>
+    <row r="100" ht="17.01" customHeight="1"/>
+    <row r="101" ht="17.01" customHeight="1"/>
+    <row r="102" ht="17.01" customHeight="1"/>
+    <row r="103" ht="17.01" customHeight="1"/>
+    <row r="104" ht="17.01" customHeight="1"/>
+    <row r="105" ht="17.01" customHeight="1"/>
+    <row r="106" ht="17.01" customHeight="1"/>
+    <row r="107" ht="17.01" customHeight="1"/>
+    <row r="108" ht="17.01" customHeight="1"/>
+    <row r="109" ht="17.01" customHeight="1"/>
+    <row r="110" ht="17.01" customHeight="1"/>
+    <row r="111" ht="17.01" customHeight="1"/>
+    <row r="112" ht="17.01" customHeight="1"/>
+    <row r="113" ht="17.01" customHeight="1"/>
+    <row r="114" ht="17.01" customHeight="1"/>
+    <row r="115" ht="17.01" customHeight="1"/>
+    <row r="116" ht="17.01" customHeight="1"/>
+    <row r="117" ht="17.01" customHeight="1"/>
+    <row r="118" ht="17.01" customHeight="1"/>
+    <row r="119" ht="17.01" customHeight="1"/>
+    <row r="120" ht="17.01" customHeight="1"/>
+    <row r="121" ht="17.01" customHeight="1"/>
+    <row r="122" ht="17.01" customHeight="1"/>
+    <row r="123" ht="17.01" customHeight="1"/>
+    <row r="124" ht="17.01" customHeight="1"/>
+    <row r="125" ht="17.01" customHeight="1"/>
+    <row r="126" ht="17.01" customHeight="1"/>
+    <row r="127" ht="17.01" customHeight="1"/>
+    <row r="128" ht="17.01" customHeight="1"/>
+    <row r="129" ht="17.01" customHeight="1"/>
+    <row r="130" ht="17.01" customHeight="1"/>
+    <row r="131" ht="17.01" customHeight="1"/>
+    <row r="132" ht="17.01" customHeight="1"/>
+    <row r="133" ht="17.01" customHeight="1"/>
+    <row r="134" ht="17.01" customHeight="1"/>
+    <row r="135" ht="17.01" customHeight="1"/>
+    <row r="136" ht="17.01" customHeight="1"/>
+    <row r="137" ht="17.01" customHeight="1"/>
+    <row r="138" ht="17.01" customHeight="1"/>
+    <row r="139" ht="17.01" customHeight="1"/>
+    <row r="140" ht="17.01" customHeight="1"/>
+    <row r="141" ht="17.01" customHeight="1"/>
+    <row r="142" ht="17.01" customHeight="1"/>
+    <row r="143" ht="17.01" customHeight="1"/>
+    <row r="144" ht="17.01" customHeight="1"/>
+    <row r="145" ht="17.01" customHeight="1"/>
+    <row r="146" ht="17.01" customHeight="1"/>
+    <row r="147" ht="17.01" customHeight="1"/>
+    <row r="148" ht="17.01" customHeight="1"/>
+    <row r="149" ht="17.01" customHeight="1"/>
+    <row r="150" ht="17.01" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.47" right="0.47" top="0.41" bottom="0.41" header="0" footer="0"/>
+  <pageMargins left="0.47" right="0.47" top="0.41" bottom="0.41" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>